<commit_message>
latest draft guidance scripts
</commit_message>
<xml_diff>
--- a/patients_overtime_100x100_post_ECM1.xlsx
+++ b/patients_overtime_100x100_post_ECM1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uob.sharepoint.com/teams/grp-Bristol_TAG-MTA-MS/Shared Documents/MTA-MS/Working Folder_HE/MS Models/Git Repo/MS-MTA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="8_{E70C0E62-E2AE-4144-9E7A-DA17AFA9C455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6873BAB6-414E-4AAC-9F29-8C42CC5B5348}"/>
+  <xr:revisionPtr revIDLastSave="123" documentId="8_{E70C0E62-E2AE-4144-9E7A-DA17AFA9C455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BE35042-06D7-44FF-9876-1F7FAD4C43B4}"/>
   <bookViews>
-    <workbookView xWindow="14595" yWindow="-16425" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{47EB86FA-01F0-49CD-AD22-F349AA4DF3BF}"/>
+    <workbookView xWindow="-10275" yWindow="-15255" windowWidth="21900" windowHeight="15915" activeTab="1" xr2:uid="{47EB86FA-01F0-49CD-AD22-F349AA4DF3BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Proportion_patients by severity" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="45">
   <si>
     <t>Jick (edss0-3) Harding (4-9)</t>
   </si>
@@ -167,6 +167,12 @@
   </si>
   <si>
     <t>distribution of patients by final edss state</t>
+  </si>
+  <si>
+    <t>Harding but not centred on Jick</t>
+  </si>
+  <si>
+    <t>Harding  centred on Jick</t>
   </si>
 </sst>
 </file>
@@ -681,10 +687,10 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -893,34 +899,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.4522319958605776E-2</c:v>
+                  <c:v>4.3369671403860457E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.8513805917493781E-2</c:v>
+                  <c:v>8.1541076758074482E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.14844889223387744</c:v>
+                  <c:v>0.1516519432253747</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.18553612587609958</c:v>
+                  <c:v>0.19037902529524056</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.20970236135283885</c:v>
+                  <c:v>0.20793064198585712</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18856719507032318</c:v>
+                  <c:v>0.18559004800927323</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.13905287172491654</c:v>
+                  <c:v>0.13413318913622144</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.5447104755632914E-3</c:v>
+                  <c:v>5.2878913263644696E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0583752763535444E-4</c:v>
+                  <c:v>1.1352535050951969E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.8798626464085812E-6</c:v>
+                  <c:v>2.9875092239347287E-6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1003,34 +1009,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.4413626237441182E-2</c:v>
+                  <c:v>4.3884554537634665E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.6924211799766912E-2</c:v>
+                  <c:v>7.6328025841689559E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.15155574571044986</c:v>
+                  <c:v>0.15138081001906845</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.18517873740428736</c:v>
+                  <c:v>0.18856433052820268</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.21130110207875366</c:v>
+                  <c:v>0.21869492249297712</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18466531918974347</c:v>
+                  <c:v>0.18241670325968612</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.14014841917351473</c:v>
+                  <c:v>0.13312440223046984</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.662353756952539E-3</c:v>
+                  <c:v>5.494968209187755E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.5048464909045312E-4</c:v>
+                  <c:v>1.0827523564901979E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>3.0076454346949944E-6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1113,31 +1119,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.6972315804892341E-2</c:v>
+                  <c:v>4.5612476971729994E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.9522484253698553E-2</c:v>
+                  <c:v>8.2103658719538189E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.14776036326351252</c:v>
+                  <c:v>0.15444393103820744</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.18710121576094918</c:v>
+                  <c:v>0.18982795556969093</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.20741467701772376</c:v>
+                  <c:v>0.21014384042534043</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18543137542112204</c:v>
+                  <c:v>0.17906842771673581</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.14017870221180609</c:v>
+                  <c:v>0.13321291623410528</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.5046140325179438E-3</c:v>
+                  <c:v>5.4427728737480733E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.1425223377764758E-4</c:v>
+                  <c:v>1.4402045090402838E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -1223,34 +1229,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.6409381004166292E-2</c:v>
+                  <c:v>4.5036831300567563E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.326457545533264E-2</c:v>
+                  <c:v>7.9286921869339444E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.15156665918347711</c:v>
+                  <c:v>0.15322424827919331</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.18426722567064441</c:v>
+                  <c:v>0.18248098055790363</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.20517447979684597</c:v>
+                  <c:v>0.20921688201907981</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18755302617269839</c:v>
+                  <c:v>0.18896570462504525</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.1363767562414174</c:v>
+                  <c:v>0.13634524815843496</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.2508666408156478E-3</c:v>
+                  <c:v>5.3163869097935029E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.3119877781049647E-4</c:v>
+                  <c:v>1.2377732157951938E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.831056791577621E-6</c:v>
+                  <c:v>3.0189590629151066E-6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1333,34 +1339,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.4039578221045213E-2</c:v>
+                  <c:v>4.5519094341474484E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.9930027454505703E-2</c:v>
+                  <c:v>7.2058864123617117E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.14505029276707401</c:v>
+                  <c:v>0.14556847493704742</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.17918924172113027</c:v>
+                  <c:v>0.18622925478240329</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.21238975679681238</c:v>
+                  <c:v>0.21403881130784966</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.19197806069146481</c:v>
+                  <c:v>0.1848766558601885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.15057156393498386</c:v>
+                  <c:v>0.1450439978039437</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6.7330353021210435E-3</c:v>
+                  <c:v>6.5176251920782474E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.1236910517748245E-4</c:v>
+                  <c:v>1.3802029818518641E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>6.0740056852693217E-6</c:v>
+                  <c:v>9.2013532123457603E-6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1443,31 +1449,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.3388629692297315E-2</c:v>
+                  <c:v>4.8803747145869755E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.7214518006750513E-2</c:v>
+                  <c:v>8.4879351890569874E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.152027353956324</c:v>
+                  <c:v>0.15973202010751689</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.19011996680458987</c:v>
+                  <c:v>0.18550718533872024</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.20713408071880379</c:v>
+                  <c:v>0.20311780826862971</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18160411247731009</c:v>
+                  <c:v>0.17794430422396237</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.14282823721228932</c:v>
+                  <c:v>0.13442314229587893</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.5658028626642542E-3</c:v>
+                  <c:v>5.4901583271412379E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.1729826897079566E-4</c:v>
+                  <c:v>1.0228240171112443E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -1555,34 +1561,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.4481102809069709E-2</c:v>
+                  <c:v>4.5605029311756376E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.9990707986720658E-2</c:v>
+                  <c:v>7.4701653529661363E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.15058942533602684</c:v>
+                  <c:v>0.1507897142925439</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1916507143970336</c:v>
+                  <c:v>0.1922325339580134</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.21037588546123379</c:v>
+                  <c:v>0.21219799329504779</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18238810622300244</c:v>
+                  <c:v>0.1832089351555824</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.13509881585640901</c:v>
+                  <c:v>0.13580516197658646</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.3458481461551351E-3</c:v>
+                  <c:v>5.3514124023688447E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7.9393784348838649E-5</c:v>
+                  <c:v>1.0159018519293172E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>5.9758932466430429E-6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2995,34 +3001,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.4522319958605776E-2</c:v>
+                  <c:v>4.3369671403860457E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.8513805917493781E-2</c:v>
+                  <c:v>8.1541076758074482E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.14844889223387744</c:v>
+                  <c:v>0.1516519432253747</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.18553612587609958</c:v>
+                  <c:v>0.19037902529524056</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.20970236135283885</c:v>
+                  <c:v>0.20793064198585712</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18856719507032318</c:v>
+                  <c:v>0.18559004800927323</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.13905287172491654</c:v>
+                  <c:v>0.13413318913622144</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.5447104755632914E-3</c:v>
+                  <c:v>5.2878913263644696E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0583752763535444E-4</c:v>
+                  <c:v>1.1352535050951969E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.8798626464085812E-6</c:v>
+                  <c:v>2.9875092239347287E-6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3454,34 +3460,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.4413626237441182E-2</c:v>
+                  <c:v>4.3884554537634665E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.6924211799766912E-2</c:v>
+                  <c:v>7.6328025841689559E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.15155574571044986</c:v>
+                  <c:v>0.15138081001906845</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.18517873740428736</c:v>
+                  <c:v>0.18856433052820268</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.21130110207875366</c:v>
+                  <c:v>0.21869492249297712</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18466531918974347</c:v>
+                  <c:v>0.18241670325968612</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.14014841917351473</c:v>
+                  <c:v>0.13312440223046984</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.662353756952539E-3</c:v>
+                  <c:v>5.494968209187755E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.5048464909045312E-4</c:v>
+                  <c:v>1.0827523564901979E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>3.0076454346949944E-6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4627,7 +4633,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -9317,43 +9323,43 @@
       <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <f>O4/$Y4</f>
         <v>2.2499999999999999E-2</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <f t="shared" ref="E4:M4" si="0">P4/$Y4</f>
         <v>6.1100000000000002E-2</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <f t="shared" si="0"/>
         <v>0.1074</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <f t="shared" si="0"/>
         <v>0.14779999999999999</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <f t="shared" si="0"/>
         <v>0.1807</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="4">
         <f t="shared" si="0"/>
         <v>0.18970000000000001</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="4">
         <f t="shared" si="0"/>
         <v>0.15179999999999999</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="4">
         <f t="shared" si="0"/>
         <v>8.7400000000000005E-2</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="4">
         <f t="shared" si="0"/>
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="4">
         <f t="shared" si="0"/>
         <v>1.11E-2</v>
       </c>
@@ -9396,43 +9402,43 @@
       <c r="C5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <f t="shared" ref="D5:D10" si="1">O5/$Y5</f>
         <v>2.2499999999999999E-2</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <f t="shared" ref="E5:E10" si="2">P5/$Y5</f>
         <v>6.1100000000000002E-2</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <f t="shared" ref="F5:F10" si="3">Q5/$Y5</f>
         <v>0.1074</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <f t="shared" ref="G5:G10" si="4">R5/$Y5</f>
         <v>0.14779999999999999</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <f t="shared" ref="H5:H10" si="5">S5/$Y5</f>
         <v>0.1807</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="4">
         <f t="shared" ref="I5:I10" si="6">T5/$Y5</f>
         <v>0.18970000000000001</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="4">
         <f t="shared" ref="J5:J10" si="7">U5/$Y5</f>
         <v>0.15179999999999999</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="4">
         <f t="shared" ref="K5:K10" si="8">V5/$Y5</f>
         <v>8.7400000000000005E-2</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="4">
         <f t="shared" ref="L5:L10" si="9">W5/$Y5</f>
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="4">
         <f t="shared" ref="M5:M10" si="10">X5/$Y5</f>
         <v>1.11E-2</v>
       </c>
@@ -9475,43 +9481,43 @@
       <c r="C6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <f t="shared" si="1"/>
         <v>2.2499999999999999E-2</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <f t="shared" si="2"/>
         <v>6.1100000000000002E-2</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <f t="shared" si="3"/>
         <v>0.1074</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <f t="shared" si="4"/>
         <v>0.14779999999999999</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="4">
         <f t="shared" si="5"/>
         <v>0.1807</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="4">
         <f t="shared" si="6"/>
         <v>0.18970000000000001</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="4">
         <f t="shared" si="7"/>
         <v>0.15179999999999999</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="4">
         <f t="shared" si="8"/>
         <v>8.7400000000000005E-2</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="4">
         <f t="shared" si="9"/>
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="4">
         <f t="shared" si="10"/>
         <v>1.11E-2</v>
       </c>
@@ -9554,43 +9560,43 @@
       <c r="C7" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <f t="shared" si="1"/>
         <v>2.2499999999999999E-2</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <f t="shared" si="2"/>
         <v>6.1100000000000002E-2</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <f t="shared" si="3"/>
         <v>0.1074</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <f t="shared" si="4"/>
         <v>0.14779999999999999</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="4">
         <f t="shared" si="5"/>
         <v>0.1807</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="4">
         <f t="shared" si="6"/>
         <v>0.18970000000000001</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="4">
         <f t="shared" si="7"/>
         <v>0.15179999999999999</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="4">
         <f t="shared" si="8"/>
         <v>8.7400000000000005E-2</v>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="4">
         <f t="shared" si="9"/>
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="4">
         <f t="shared" si="10"/>
         <v>1.11E-2</v>
       </c>
@@ -9633,43 +9639,43 @@
       <c r="C8" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <f t="shared" si="1"/>
         <v>2.2499999999999999E-2</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <f t="shared" si="2"/>
         <v>6.1100000000000002E-2</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="4">
         <f t="shared" si="3"/>
         <v>0.1074</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <f t="shared" si="4"/>
         <v>0.14779999999999999</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="4">
         <f t="shared" si="5"/>
         <v>0.1807</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="4">
         <f t="shared" si="6"/>
         <v>0.18970000000000001</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="4">
         <f t="shared" si="7"/>
         <v>0.15179999999999999</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="4">
         <f t="shared" si="8"/>
         <v>8.7400000000000005E-2</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="4">
         <f t="shared" si="9"/>
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="4">
         <f t="shared" si="10"/>
         <v>1.11E-2</v>
       </c>
@@ -9712,43 +9718,43 @@
       <c r="C9" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <f t="shared" si="1"/>
         <v>2.2499999999999999E-2</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="4">
         <f t="shared" si="2"/>
         <v>6.1100000000000002E-2</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="4">
         <f t="shared" si="3"/>
         <v>0.1074</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <f t="shared" si="4"/>
         <v>0.14779999999999999</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="4">
         <f t="shared" si="5"/>
         <v>0.1807</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="4">
         <f t="shared" si="6"/>
         <v>0.18970000000000001</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="4">
         <f t="shared" si="7"/>
         <v>0.15179999999999999</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="4">
         <f t="shared" si="8"/>
         <v>8.7400000000000005E-2</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="4">
         <f t="shared" si="9"/>
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="4">
         <f t="shared" si="10"/>
         <v>1.11E-2</v>
       </c>
@@ -9791,43 +9797,43 @@
       <c r="C10" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
         <f t="shared" si="1"/>
         <v>2.2499999999999999E-2</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <f t="shared" si="2"/>
         <v>6.1100000000000002E-2</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="4">
         <f t="shared" si="3"/>
         <v>0.1074</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <f t="shared" si="4"/>
         <v>0.14779999999999999</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="4">
         <f t="shared" si="5"/>
         <v>0.1807</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="4">
         <f t="shared" si="6"/>
         <v>0.18970000000000001</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="4">
         <f t="shared" si="7"/>
         <v>0.15179999999999999</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="4">
         <f t="shared" si="8"/>
         <v>8.7400000000000005E-2</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="4">
         <f t="shared" si="9"/>
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="4">
         <f t="shared" si="10"/>
         <v>1.11E-2</v>
       </c>
@@ -9935,43 +9941,43 @@
       <c r="C14" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="4">
         <f>O14/$Y14</f>
         <v>0.02</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="4">
         <f t="shared" ref="E14:E20" si="12">P14/$Y14</f>
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="4">
         <f t="shared" ref="F14:F20" si="13">Q14/$Y14</f>
         <v>0.1007</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="4">
         <f t="shared" ref="G14:G20" si="14">R14/$Y14</f>
         <v>0.15579999999999999</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="4">
         <f t="shared" ref="H14:H20" si="15">S14/$Y14</f>
         <v>0.18790000000000001</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="4">
         <f t="shared" ref="I14:I20" si="16">T14/$Y14</f>
         <v>0.18740000000000001</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="4">
         <f t="shared" ref="J14:J20" si="17">U14/$Y14</f>
         <v>0.1595</v>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="4">
         <f t="shared" ref="K14:K20" si="18">V14/$Y14</f>
         <v>8.77E-2</v>
       </c>
-      <c r="L14" s="5">
+      <c r="L14" s="4">
         <f t="shared" ref="L14:L20" si="19">W14/$Y14</f>
         <v>3.4500000000000003E-2</v>
       </c>
-      <c r="M14" s="5">
+      <c r="M14" s="4">
         <f t="shared" ref="M14:M20" si="20">X14/$Y14</f>
         <v>1.09E-2</v>
       </c>
@@ -10014,43 +10020,43 @@
       <c r="C15" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="4">
         <f t="shared" ref="D15:D20" si="21">O15/$Y15</f>
         <v>0.02</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="4">
         <f t="shared" si="12"/>
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="4">
         <f t="shared" si="13"/>
         <v>0.1007</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="4">
         <f t="shared" si="14"/>
         <v>0.15579999999999999</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="4">
         <f t="shared" si="15"/>
         <v>0.18790000000000001</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="4">
         <f t="shared" si="16"/>
         <v>0.18740000000000001</v>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="4">
         <f t="shared" si="17"/>
         <v>0.1595</v>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="4">
         <f t="shared" si="18"/>
         <v>8.77E-2</v>
       </c>
-      <c r="L15" s="5">
+      <c r="L15" s="4">
         <f t="shared" si="19"/>
         <v>3.4500000000000003E-2</v>
       </c>
-      <c r="M15" s="5">
+      <c r="M15" s="4">
         <f t="shared" si="20"/>
         <v>1.09E-2</v>
       </c>
@@ -10093,43 +10099,43 @@
       <c r="C16" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="4">
         <f t="shared" si="21"/>
         <v>0.02</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="4">
         <f t="shared" si="12"/>
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="4">
         <f t="shared" si="13"/>
         <v>0.1007</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="4">
         <f t="shared" si="14"/>
         <v>0.15579999999999999</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="4">
         <f t="shared" si="15"/>
         <v>0.18790000000000001</v>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="4">
         <f t="shared" si="16"/>
         <v>0.18740000000000001</v>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="4">
         <f t="shared" si="17"/>
         <v>0.1595</v>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="4">
         <f t="shared" si="18"/>
         <v>8.77E-2</v>
       </c>
-      <c r="L16" s="5">
+      <c r="L16" s="4">
         <f t="shared" si="19"/>
         <v>3.4500000000000003E-2</v>
       </c>
-      <c r="M16" s="5">
+      <c r="M16" s="4">
         <f t="shared" si="20"/>
         <v>1.09E-2</v>
       </c>
@@ -10172,43 +10178,43 @@
       <c r="C17" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="4">
         <f t="shared" si="21"/>
         <v>0.02</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="4">
         <f t="shared" si="12"/>
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="4">
         <f t="shared" si="13"/>
         <v>0.1007</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="4">
         <f t="shared" si="14"/>
         <v>0.15579999999999999</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="4">
         <f t="shared" si="15"/>
         <v>0.18790000000000001</v>
       </c>
-      <c r="I17" s="5">
+      <c r="I17" s="4">
         <f t="shared" si="16"/>
         <v>0.18740000000000001</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="4">
         <f t="shared" si="17"/>
         <v>0.1595</v>
       </c>
-      <c r="K17" s="5">
+      <c r="K17" s="4">
         <f t="shared" si="18"/>
         <v>8.77E-2</v>
       </c>
-      <c r="L17" s="5">
+      <c r="L17" s="4">
         <f t="shared" si="19"/>
         <v>3.4500000000000003E-2</v>
       </c>
-      <c r="M17" s="5">
+      <c r="M17" s="4">
         <f t="shared" si="20"/>
         <v>1.09E-2</v>
       </c>
@@ -10251,43 +10257,43 @@
       <c r="C18" t="s">
         <v>15</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="4">
         <f t="shared" si="21"/>
         <v>0.02</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="4">
         <f t="shared" si="12"/>
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="4">
         <f t="shared" si="13"/>
         <v>0.1007</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="4">
         <f t="shared" si="14"/>
         <v>0.15579999999999999</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="4">
         <f t="shared" si="15"/>
         <v>0.18790000000000001</v>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="4">
         <f t="shared" si="16"/>
         <v>0.18740000000000001</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="4">
         <f t="shared" si="17"/>
         <v>0.1595</v>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="4">
         <f t="shared" si="18"/>
         <v>8.77E-2</v>
       </c>
-      <c r="L18" s="5">
+      <c r="L18" s="4">
         <f t="shared" si="19"/>
         <v>3.4500000000000003E-2</v>
       </c>
-      <c r="M18" s="5">
+      <c r="M18" s="4">
         <f t="shared" si="20"/>
         <v>1.09E-2</v>
       </c>
@@ -10330,43 +10336,43 @@
       <c r="C19" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="4">
         <f t="shared" si="21"/>
         <v>0.02</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="4">
         <f t="shared" si="12"/>
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="4">
         <f t="shared" si="13"/>
         <v>0.1007</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="4">
         <f t="shared" si="14"/>
         <v>0.15579999999999999</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="4">
         <f t="shared" si="15"/>
         <v>0.18790000000000001</v>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="4">
         <f t="shared" si="16"/>
         <v>0.18740000000000001</v>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="4">
         <f t="shared" si="17"/>
         <v>0.1595</v>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="4">
         <f t="shared" si="18"/>
         <v>8.77E-2</v>
       </c>
-      <c r="L19" s="5">
+      <c r="L19" s="4">
         <f t="shared" si="19"/>
         <v>3.4500000000000003E-2</v>
       </c>
-      <c r="M19" s="5">
+      <c r="M19" s="4">
         <f t="shared" si="20"/>
         <v>1.09E-2</v>
       </c>
@@ -10409,43 +10415,43 @@
       <c r="C20" t="s">
         <v>17</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="4">
         <f t="shared" si="21"/>
         <v>0.02</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="4">
         <f t="shared" si="12"/>
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="4">
         <f t="shared" si="13"/>
         <v>0.1007</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="4">
         <f t="shared" si="14"/>
         <v>0.15579999999999999</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="4">
         <f t="shared" si="15"/>
         <v>0.18790000000000001</v>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="4">
         <f t="shared" si="16"/>
         <v>0.18740000000000001</v>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="4">
         <f t="shared" si="17"/>
         <v>0.1595</v>
       </c>
-      <c r="K20" s="5">
+      <c r="K20" s="4">
         <f t="shared" si="18"/>
         <v>8.77E-2</v>
       </c>
-      <c r="L20" s="5">
+      <c r="L20" s="4">
         <f t="shared" si="19"/>
         <v>3.4500000000000003E-2</v>
       </c>
-      <c r="M20" s="5">
+      <c r="M20" s="4">
         <f t="shared" si="20"/>
         <v>1.09E-2</v>
       </c>
@@ -10491,28 +10497,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E5FF2E5-E9BF-445B-9A93-EBCF9FC87E4A}">
-  <dimension ref="A1:X17"/>
+  <dimension ref="A1:AJ17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.88671875" customWidth="1"/>
     <col min="2" max="11" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="B1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -10546,212 +10552,286 @@
       <c r="K2" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="N2" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3">
         <f>N3/$X3</f>
-        <v>4.4522319958605776E-2</v>
+        <v>4.3369671403860457E-2</v>
       </c>
       <c r="C3">
         <f t="shared" ref="C3:K3" si="0">O3/$X3</f>
-        <v>7.8513805917493781E-2</v>
+        <v>8.1541076758074482E-2</v>
       </c>
       <c r="D3">
         <f t="shared" si="0"/>
-        <v>0.14844889223387744</v>
+        <v>0.1516519432253747</v>
       </c>
       <c r="E3">
         <f t="shared" si="0"/>
-        <v>0.18553612587609958</v>
+        <v>0.19037902529524056</v>
       </c>
       <c r="F3">
         <f t="shared" si="0"/>
-        <v>0.20970236135283885</v>
+        <v>0.20793064198585712</v>
       </c>
       <c r="G3">
         <f t="shared" si="0"/>
-        <v>0.18856719507032318</v>
+        <v>0.18559004800927323</v>
       </c>
       <c r="H3">
         <f t="shared" si="0"/>
-        <v>0.13905287172491654</v>
+        <v>0.13413318913622144</v>
       </c>
       <c r="I3">
         <f t="shared" si="0"/>
-        <v>5.5447104755632914E-3</v>
+        <v>5.2878913263644696E-3</v>
       </c>
       <c r="J3">
         <f t="shared" si="0"/>
-        <v>1.0583752763535444E-4</v>
+        <v>1.1352535050951969E-4</v>
       </c>
       <c r="K3">
         <f t="shared" si="0"/>
-        <v>5.8798626464085812E-6</v>
+        <v>2.9875092239347287E-6</v>
       </c>
       <c r="L3">
         <f>SUM(B3:K3)</f>
-        <v>1.0000000000000002</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="N3">
-        <v>1.5144</v>
+        <v>1.4517</v>
       </c>
       <c r="O3">
-        <v>2.6705999999999999</v>
+        <v>2.7294</v>
       </c>
       <c r="P3">
-        <v>5.0494000000000003</v>
+        <v>5.0762</v>
       </c>
       <c r="Q3">
-        <v>6.3109000000000002</v>
+        <v>6.3724999999999996</v>
       </c>
       <c r="R3">
-        <v>7.1329000000000002</v>
+        <v>6.96</v>
       </c>
       <c r="S3">
-        <v>6.4139999999999997</v>
+        <v>6.2122000000000002</v>
       </c>
       <c r="T3">
-        <v>4.7298</v>
+        <v>4.4897999999999998</v>
       </c>
       <c r="U3">
-        <v>0.18859999999999999</v>
+        <v>0.17699999999999999</v>
       </c>
       <c r="V3">
-        <v>3.5999999999999999E-3</v>
+        <v>3.8E-3</v>
       </c>
       <c r="W3">
-        <v>2.0000000000000001E-4</v>
+        <v>1E-4</v>
       </c>
       <c r="X3">
         <f>SUM(N3:W3)</f>
+        <v>33.472700000000003</v>
+      </c>
+      <c r="Z3">
+        <v>1.5144</v>
+      </c>
+      <c r="AA3">
+        <v>2.6705999999999999</v>
+      </c>
+      <c r="AB3">
+        <v>5.0494000000000003</v>
+      </c>
+      <c r="AC3">
+        <v>6.3109000000000002</v>
+      </c>
+      <c r="AD3">
+        <v>7.1329000000000002</v>
+      </c>
+      <c r="AE3">
+        <v>6.4139999999999997</v>
+      </c>
+      <c r="AF3">
+        <v>4.7298</v>
+      </c>
+      <c r="AG3">
+        <v>0.18859999999999999</v>
+      </c>
+      <c r="AH3">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="AI3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="AJ3">
+        <f>SUM(Z3:AI3)</f>
         <v>34.014399999999995</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:B9" si="1">N4/$X4</f>
-        <v>4.4413626237441182E-2</v>
+        <v>4.3884554537634665E-2</v>
       </c>
       <c r="C4">
         <f t="shared" ref="C4:C9" si="2">O4/$X4</f>
-        <v>7.6924211799766912E-2</v>
+        <v>7.6328025841689559E-2</v>
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D9" si="3">P4/$X4</f>
-        <v>0.15155574571044986</v>
+        <v>0.15138081001906845</v>
       </c>
       <c r="E4">
         <f t="shared" ref="E4:E9" si="4">Q4/$X4</f>
-        <v>0.18517873740428736</v>
+        <v>0.18856433052820268</v>
       </c>
       <c r="F4">
         <f t="shared" ref="F4:F9" si="5">R4/$X4</f>
-        <v>0.21130110207875366</v>
+        <v>0.21869492249297712</v>
       </c>
       <c r="G4">
         <f t="shared" ref="G4:G9" si="6">S4/$X4</f>
-        <v>0.18466531918974347</v>
+        <v>0.18241670325968612</v>
       </c>
       <c r="H4">
         <f t="shared" ref="H4:H9" si="7">T4/$X4</f>
-        <v>0.14014841917351473</v>
+        <v>0.13312440223046984</v>
       </c>
       <c r="I4">
         <f t="shared" ref="I4:I9" si="8">U4/$X4</f>
-        <v>5.662353756952539E-3</v>
+        <v>5.494968209187755E-3</v>
       </c>
       <c r="J4">
         <f t="shared" ref="J4:J9" si="9">V4/$X4</f>
-        <v>1.5048464909045312E-4</v>
+        <v>1.0827523564901979E-4</v>
       </c>
       <c r="K4">
         <f t="shared" ref="K4:K9" si="10">W4/$X4</f>
-        <v>0</v>
+        <v>3.0076454346949944E-6</v>
       </c>
       <c r="L4">
         <f t="shared" ref="L4:L9" si="11">SUM(B4:K4)</f>
-        <v>1.0000000000000002</v>
+        <v>1</v>
       </c>
       <c r="N4">
-        <v>1.5052000000000001</v>
+        <v>1.4591000000000001</v>
       </c>
       <c r="O4">
-        <v>2.6070000000000002</v>
+        <v>2.5377999999999998</v>
       </c>
       <c r="P4">
-        <v>5.1363000000000003</v>
+        <v>5.0331999999999999</v>
       </c>
       <c r="Q4">
-        <v>6.2758000000000003</v>
+        <v>6.2694999999999999</v>
       </c>
       <c r="R4">
-        <v>7.1611000000000002</v>
+        <v>7.2713000000000001</v>
       </c>
       <c r="S4">
-        <v>6.2584</v>
+        <v>6.0651000000000002</v>
       </c>
       <c r="T4">
-        <v>4.7496999999999998</v>
+        <v>4.4261999999999997</v>
       </c>
       <c r="U4">
-        <v>0.19189999999999999</v>
+        <v>0.1827</v>
       </c>
       <c r="V4">
-        <v>5.1000000000000004E-3</v>
+        <v>3.5999999999999999E-3</v>
       </c>
       <c r="W4">
-        <v>0</v>
+        <v>1E-4</v>
       </c>
       <c r="X4">
         <f t="shared" ref="X4:X9" si="12">SUM(N4:W4)</f>
+        <v>33.248600000000003</v>
+      </c>
+      <c r="Z4">
+        <v>1.5052000000000001</v>
+      </c>
+      <c r="AA4">
+        <v>2.6070000000000002</v>
+      </c>
+      <c r="AB4">
+        <v>5.1363000000000003</v>
+      </c>
+      <c r="AC4">
+        <v>6.2758000000000003</v>
+      </c>
+      <c r="AD4">
+        <v>7.1611000000000002</v>
+      </c>
+      <c r="AE4">
+        <v>6.2584</v>
+      </c>
+      <c r="AF4">
+        <v>4.7496999999999998</v>
+      </c>
+      <c r="AG4">
+        <v>0.19189999999999999</v>
+      </c>
+      <c r="AH4">
+        <v>5.1000000000000004E-3</v>
+      </c>
+      <c r="AI4">
+        <v>0</v>
+      </c>
+      <c r="AJ4">
+        <f t="shared" ref="AJ4:AJ9" si="13">SUM(Z4:AI4)</f>
         <v>33.890499999999996</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5">
         <f t="shared" si="1"/>
-        <v>4.6972315804892341E-2</v>
+        <v>4.5612476971729994E-2</v>
       </c>
       <c r="C5">
         <f t="shared" si="2"/>
-        <v>7.9522484253698553E-2</v>
+        <v>8.2103658719538189E-2</v>
       </c>
       <c r="D5">
         <f t="shared" si="3"/>
-        <v>0.14776036326351252</v>
+        <v>0.15444393103820744</v>
       </c>
       <c r="E5">
         <f t="shared" si="4"/>
-        <v>0.18710121576094918</v>
+        <v>0.18982795556969093</v>
       </c>
       <c r="F5">
         <f t="shared" si="5"/>
-        <v>0.20741467701772376</v>
+        <v>0.21014384042534043</v>
       </c>
       <c r="G5">
         <f t="shared" si="6"/>
-        <v>0.18543137542112204</v>
+        <v>0.17906842771673581</v>
       </c>
       <c r="H5">
         <f t="shared" si="7"/>
-        <v>0.14017870221180609</v>
+        <v>0.13321291623410528</v>
       </c>
       <c r="I5">
         <f t="shared" si="8"/>
-        <v>5.5046140325179438E-3</v>
+        <v>5.4427728737480733E-3</v>
       </c>
       <c r="J5">
         <f t="shared" si="9"/>
-        <v>1.1425223377764758E-4</v>
+        <v>1.4402045090402838E-4</v>
       </c>
       <c r="K5">
         <f t="shared" si="10"/>
@@ -10759,248 +10839,350 @@
       </c>
       <c r="L5">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="N5">
-        <v>1.6033999999999999</v>
+        <v>1.5202</v>
       </c>
       <c r="O5">
-        <v>2.7145000000000001</v>
+        <v>2.7364000000000002</v>
       </c>
       <c r="P5">
-        <v>5.0438000000000001</v>
+        <v>5.1474000000000002</v>
       </c>
       <c r="Q5">
-        <v>6.3867000000000003</v>
+        <v>6.3266999999999998</v>
       </c>
       <c r="R5">
-        <v>7.0800999999999998</v>
+        <v>7.0038</v>
       </c>
       <c r="S5">
-        <v>6.3296999999999999</v>
+        <v>5.9680999999999997</v>
       </c>
       <c r="T5">
-        <v>4.7850000000000001</v>
+        <v>4.4398</v>
       </c>
       <c r="U5">
-        <v>0.18790000000000001</v>
+        <v>0.18140000000000001</v>
       </c>
       <c r="V5">
-        <v>3.8999999999999998E-3</v>
+        <v>4.7999999999999996E-3</v>
       </c>
       <c r="W5">
         <v>0</v>
       </c>
       <c r="X5">
         <f t="shared" si="12"/>
+        <v>33.328599999999994</v>
+      </c>
+      <c r="Z5">
+        <v>1.6033999999999999</v>
+      </c>
+      <c r="AA5">
+        <v>2.7145000000000001</v>
+      </c>
+      <c r="AB5">
+        <v>5.0438000000000001</v>
+      </c>
+      <c r="AC5">
+        <v>6.3867000000000003</v>
+      </c>
+      <c r="AD5">
+        <v>7.0800999999999998</v>
+      </c>
+      <c r="AE5">
+        <v>6.3296999999999999</v>
+      </c>
+      <c r="AF5">
+        <v>4.7850000000000001</v>
+      </c>
+      <c r="AG5">
+        <v>0.18790000000000001</v>
+      </c>
+      <c r="AH5">
+        <v>3.8999999999999998E-3</v>
+      </c>
+      <c r="AI5">
+        <v>0</v>
+      </c>
+      <c r="AJ5">
+        <f t="shared" si="13"/>
         <v>34.134999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6">
         <f t="shared" si="1"/>
-        <v>4.6409381004166292E-2</v>
+        <v>4.5036831300567563E-2</v>
       </c>
       <c r="C6">
         <f t="shared" si="2"/>
-        <v>8.326457545533264E-2</v>
+        <v>7.9286921869339444E-2</v>
       </c>
       <c r="D6">
         <f t="shared" si="3"/>
-        <v>0.15156665918347711</v>
+        <v>0.15322424827919331</v>
       </c>
       <c r="E6">
         <f t="shared" si="4"/>
-        <v>0.18426722567064441</v>
+        <v>0.18248098055790363</v>
       </c>
       <c r="F6">
         <f t="shared" si="5"/>
-        <v>0.20517447979684597</v>
+        <v>0.20921688201907981</v>
       </c>
       <c r="G6">
         <f t="shared" si="6"/>
-        <v>0.18755302617269839</v>
+        <v>0.18896570462504525</v>
       </c>
       <c r="H6">
         <f t="shared" si="7"/>
-        <v>0.1363767562414174</v>
+        <v>0.13634524815843496</v>
       </c>
       <c r="I6">
         <f t="shared" si="8"/>
-        <v>5.2508666408156478E-3</v>
+        <v>5.3163869097935029E-3</v>
       </c>
       <c r="J6">
         <f t="shared" si="9"/>
-        <v>1.3119877781049647E-4</v>
+        <v>1.2377732157951938E-4</v>
       </c>
       <c r="K6">
         <f t="shared" si="10"/>
-        <v>5.831056791577621E-6</v>
+        <v>3.0189590629151066E-6</v>
       </c>
       <c r="L6">
         <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="N6">
-        <v>1.5918000000000001</v>
+        <v>1.4918</v>
       </c>
       <c r="O6">
-        <v>2.8559000000000001</v>
+        <v>2.6263000000000001</v>
       </c>
       <c r="P6">
-        <v>5.1985999999999999</v>
+        <v>5.0754000000000001</v>
       </c>
       <c r="Q6">
-        <v>6.3201999999999998</v>
+        <v>6.0445000000000002</v>
       </c>
       <c r="R6">
-        <v>7.0373000000000001</v>
+        <v>6.9301000000000004</v>
       </c>
       <c r="S6">
-        <v>6.4329000000000001</v>
+        <v>6.2592999999999996</v>
       </c>
       <c r="T6">
-        <v>4.6776</v>
+        <v>4.5163000000000002</v>
       </c>
       <c r="U6">
-        <v>0.18010000000000001</v>
+        <v>0.17610000000000001</v>
       </c>
       <c r="V6">
-        <v>4.4999999999999997E-3</v>
+        <v>4.1000000000000003E-3</v>
       </c>
       <c r="W6">
-        <v>2.0000000000000001E-4</v>
+        <v>1E-4</v>
       </c>
       <c r="X6">
         <f t="shared" si="12"/>
+        <v>33.124000000000002</v>
+      </c>
+      <c r="Z6">
+        <v>1.5918000000000001</v>
+      </c>
+      <c r="AA6">
+        <v>2.8559000000000001</v>
+      </c>
+      <c r="AB6">
+        <v>5.1985999999999999</v>
+      </c>
+      <c r="AC6">
+        <v>6.3201999999999998</v>
+      </c>
+      <c r="AD6">
+        <v>7.0373000000000001</v>
+      </c>
+      <c r="AE6">
+        <v>6.4329000000000001</v>
+      </c>
+      <c r="AF6">
+        <v>4.6776</v>
+      </c>
+      <c r="AG6">
+        <v>0.18010000000000001</v>
+      </c>
+      <c r="AH6">
+        <v>4.4999999999999997E-3</v>
+      </c>
+      <c r="AI6">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="AJ6">
+        <f t="shared" si="13"/>
         <v>34.299100000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>15</v>
       </c>
       <c r="B7">
         <f t="shared" si="1"/>
-        <v>4.4039578221045213E-2</v>
+        <v>4.5519094341474484E-2</v>
       </c>
       <c r="C7">
         <f t="shared" si="2"/>
-        <v>6.9930027454505703E-2</v>
+        <v>7.2058864123617117E-2</v>
       </c>
       <c r="D7">
         <f t="shared" si="3"/>
-        <v>0.14505029276707401</v>
+        <v>0.14556847493704742</v>
       </c>
       <c r="E7">
         <f t="shared" si="4"/>
-        <v>0.17918924172113027</v>
+        <v>0.18622925478240329</v>
       </c>
       <c r="F7">
         <f t="shared" si="5"/>
-        <v>0.21238975679681238</v>
+        <v>0.21403881130784966</v>
       </c>
       <c r="G7">
         <f t="shared" si="6"/>
-        <v>0.19197806069146481</v>
+        <v>0.1848766558601885</v>
       </c>
       <c r="H7">
         <f t="shared" si="7"/>
-        <v>0.15057156393498386</v>
+        <v>0.1450439978039437</v>
       </c>
       <c r="I7">
         <f t="shared" si="8"/>
-        <v>6.7330353021210435E-3</v>
+        <v>6.5176251920782474E-3</v>
       </c>
       <c r="J7">
         <f t="shared" si="9"/>
-        <v>1.1236910517748245E-4</v>
+        <v>1.3802029818518641E-4</v>
       </c>
       <c r="K7">
         <f t="shared" si="10"/>
-        <v>6.0740056852693217E-6</v>
+        <v>9.2013532123457603E-6</v>
       </c>
       <c r="L7">
         <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="N7">
-        <v>1.4500999999999999</v>
+        <v>1.4841</v>
       </c>
       <c r="O7">
-        <v>2.3026</v>
+        <v>2.3494000000000002</v>
       </c>
       <c r="P7">
-        <v>4.7760999999999996</v>
+        <v>4.7461000000000002</v>
       </c>
       <c r="Q7">
-        <v>5.9001999999999999</v>
+        <v>6.0717999999999996</v>
       </c>
       <c r="R7">
-        <v>6.9934000000000003</v>
+        <v>6.9785000000000004</v>
       </c>
       <c r="S7">
-        <v>6.3212999999999999</v>
+        <v>6.0277000000000003</v>
       </c>
       <c r="T7">
-        <v>4.9579000000000004</v>
+        <v>4.7290000000000001</v>
       </c>
       <c r="U7">
-        <v>0.22170000000000001</v>
+        <v>0.21249999999999999</v>
       </c>
       <c r="V7">
-        <v>3.7000000000000002E-3</v>
+        <v>4.4999999999999997E-3</v>
       </c>
       <c r="W7">
-        <v>2.0000000000000001E-4</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="X7">
         <f t="shared" si="12"/>
+        <v>32.603900000000003</v>
+      </c>
+      <c r="Z7">
+        <v>1.4500999999999999</v>
+      </c>
+      <c r="AA7">
+        <v>2.3026</v>
+      </c>
+      <c r="AB7">
+        <v>4.7760999999999996</v>
+      </c>
+      <c r="AC7">
+        <v>5.9001999999999999</v>
+      </c>
+      <c r="AD7">
+        <v>6.9934000000000003</v>
+      </c>
+      <c r="AE7">
+        <v>6.3212999999999999</v>
+      </c>
+      <c r="AF7">
+        <v>4.9579000000000004</v>
+      </c>
+      <c r="AG7">
+        <v>0.22170000000000001</v>
+      </c>
+      <c r="AH7">
+        <v>3.7000000000000002E-3</v>
+      </c>
+      <c r="AI7">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="AJ7">
+        <f t="shared" si="13"/>
         <v>32.927199999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
       <c r="B8">
         <f t="shared" si="1"/>
-        <v>4.3388629692297315E-2</v>
+        <v>4.8803747145869755E-2</v>
       </c>
       <c r="C8">
         <f t="shared" si="2"/>
-        <v>7.7214518006750513E-2</v>
+        <v>8.4879351890569874E-2</v>
       </c>
       <c r="D8">
         <f t="shared" si="3"/>
-        <v>0.152027353956324</v>
+        <v>0.15973202010751689</v>
       </c>
       <c r="E8">
         <f t="shared" si="4"/>
-        <v>0.19011996680458987</v>
+        <v>0.18550718533872024</v>
       </c>
       <c r="F8">
         <f t="shared" si="5"/>
-        <v>0.20713408071880379</v>
+        <v>0.20311780826862971</v>
       </c>
       <c r="G8">
         <f t="shared" si="6"/>
-        <v>0.18160411247731009</v>
+        <v>0.17794430422396237</v>
       </c>
       <c r="H8">
         <f t="shared" si="7"/>
-        <v>0.14282823721228932</v>
+        <v>0.13442314229587893</v>
       </c>
       <c r="I8">
         <f t="shared" si="8"/>
-        <v>5.5658028626642542E-3</v>
+        <v>5.4901583271412379E-3</v>
       </c>
       <c r="J8">
         <f t="shared" si="9"/>
-        <v>1.1729826897079566E-4</v>
+        <v>1.0228240171112443E-4</v>
       </c>
       <c r="K8">
         <f t="shared" si="10"/>
@@ -11008,127 +11190,195 @@
       </c>
       <c r="L8">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="N8">
-        <v>1.4796</v>
+        <v>1.6223000000000001</v>
       </c>
       <c r="O8">
-        <v>2.6331000000000002</v>
+        <v>2.8214999999999999</v>
       </c>
       <c r="P8">
-        <v>5.1843000000000004</v>
+        <v>5.3097000000000003</v>
       </c>
       <c r="Q8">
-        <v>6.4832999999999998</v>
+        <v>6.1665000000000001</v>
       </c>
       <c r="R8">
-        <v>7.0635000000000003</v>
+        <v>6.7519</v>
       </c>
       <c r="S8">
-        <v>6.1928999999999998</v>
+        <v>5.9150999999999998</v>
       </c>
       <c r="T8">
-        <v>4.8705999999999996</v>
+        <v>4.4683999999999999</v>
       </c>
       <c r="U8">
-        <v>0.1898</v>
+        <v>0.1825</v>
       </c>
       <c r="V8">
-        <v>4.0000000000000001E-3</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="W8">
         <v>0</v>
       </c>
       <c r="X8">
         <f t="shared" si="12"/>
+        <v>33.241299999999995</v>
+      </c>
+      <c r="Z8">
+        <v>1.4796</v>
+      </c>
+      <c r="AA8">
+        <v>2.6331000000000002</v>
+      </c>
+      <c r="AB8">
+        <v>5.1843000000000004</v>
+      </c>
+      <c r="AC8">
+        <v>6.4832999999999998</v>
+      </c>
+      <c r="AD8">
+        <v>7.0635000000000003</v>
+      </c>
+      <c r="AE8">
+        <v>6.1928999999999998</v>
+      </c>
+      <c r="AF8">
+        <v>4.8705999999999996</v>
+      </c>
+      <c r="AG8">
+        <v>0.1898</v>
+      </c>
+      <c r="AH8">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="AI8">
+        <v>0</v>
+      </c>
+      <c r="AJ8">
+        <f t="shared" si="13"/>
         <v>34.101100000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B9">
         <f t="shared" si="1"/>
-        <v>4.4481102809069709E-2</v>
+        <v>4.5605029311756376E-2</v>
       </c>
       <c r="C9">
         <f t="shared" si="2"/>
-        <v>7.9990707986720658E-2</v>
+        <v>7.4701653529661363E-2</v>
       </c>
       <c r="D9">
         <f t="shared" si="3"/>
-        <v>0.15058942533602684</v>
+        <v>0.1507897142925439</v>
       </c>
       <c r="E9">
         <f t="shared" si="4"/>
-        <v>0.1916507143970336</v>
+        <v>0.1922325339580134</v>
       </c>
       <c r="F9">
         <f t="shared" si="5"/>
-        <v>0.21037588546123379</v>
+        <v>0.21219799329504779</v>
       </c>
       <c r="G9">
         <f t="shared" si="6"/>
-        <v>0.18238810622300244</v>
+        <v>0.1832089351555824</v>
       </c>
       <c r="H9">
         <f t="shared" si="7"/>
-        <v>0.13509881585640901</v>
+        <v>0.13580516197658646</v>
       </c>
       <c r="I9">
         <f t="shared" si="8"/>
-        <v>5.3458481461551351E-3</v>
+        <v>5.3514124023688447E-3</v>
       </c>
       <c r="J9">
         <f t="shared" si="9"/>
-        <v>7.9393784348838649E-5</v>
+        <v>1.0159018519293172E-4</v>
       </c>
       <c r="K9">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>5.9758932466430429E-6</v>
       </c>
       <c r="L9">
         <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="N9" s="2">
-        <v>1.5126999999999999</v>
+        <v>1.5263</v>
       </c>
       <c r="O9" s="2">
-        <v>2.7202999999999999</v>
+        <v>2.5001000000000002</v>
       </c>
       <c r="P9" s="2">
-        <v>5.1212</v>
+        <v>5.0465999999999998</v>
       </c>
       <c r="Q9" s="2">
-        <v>6.5175999999999998</v>
+        <v>6.4336000000000002</v>
       </c>
       <c r="R9" s="2">
-        <v>7.1543999999999999</v>
+        <v>7.1017999999999999</v>
       </c>
       <c r="S9" s="2">
-        <v>6.2026000000000003</v>
+        <v>6.1315999999999997</v>
       </c>
       <c r="T9" s="2">
-        <v>4.5944000000000003</v>
+        <v>4.5450999999999997</v>
       </c>
       <c r="U9" s="2">
-        <v>0.18179999999999999</v>
+        <v>0.17910000000000001</v>
       </c>
       <c r="V9" s="2">
-        <v>2.7000000000000001E-3</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="W9" s="2">
-        <v>0</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="X9">
         <f t="shared" si="12"/>
+        <v>33.467799999999997</v>
+      </c>
+      <c r="Z9" s="2">
+        <v>1.5126999999999999</v>
+      </c>
+      <c r="AA9" s="2">
+        <v>2.7202999999999999</v>
+      </c>
+      <c r="AB9" s="2">
+        <v>5.1212</v>
+      </c>
+      <c r="AC9" s="2">
+        <v>6.5175999999999998</v>
+      </c>
+      <c r="AD9" s="2">
+        <v>7.1543999999999999</v>
+      </c>
+      <c r="AE9" s="2">
+        <v>6.2026000000000003</v>
+      </c>
+      <c r="AF9" s="2">
+        <v>4.5944000000000003</v>
+      </c>
+      <c r="AG9" s="2">
+        <v>0.18179999999999999</v>
+      </c>
+      <c r="AH9" s="2">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="AI9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AJ9">
+        <f t="shared" si="13"/>
         <v>34.0077</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -11193,7 +11443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -11202,39 +11452,39 @@
         <v>3.9467507209442698E-2</v>
       </c>
       <c r="C11">
-        <f t="shared" ref="C11:C17" si="13">O11/$X11</f>
+        <f t="shared" ref="C11:C17" si="14">O11/$X11</f>
         <v>7.0582679453647199E-2</v>
       </c>
       <c r="D11">
-        <f t="shared" ref="D11:D17" si="14">P11/$X11</f>
+        <f t="shared" ref="D11:D17" si="15">P11/$X11</f>
         <v>0.14286153399056625</v>
       </c>
       <c r="E11">
-        <f t="shared" ref="E11:E17" si="15">Q11/$X11</f>
+        <f t="shared" ref="E11:E17" si="16">Q11/$X11</f>
         <v>0.18743433259562292</v>
       </c>
       <c r="F11">
-        <f t="shared" ref="F11:F17" si="16">R11/$X11</f>
+        <f t="shared" ref="F11:F17" si="17">R11/$X11</f>
         <v>0.21587251022734893</v>
       </c>
       <c r="G11">
-        <f t="shared" ref="G11:G17" si="17">S11/$X11</f>
+        <f t="shared" ref="G11:G17" si="18">S11/$X11</f>
         <v>0.19193045402722822</v>
       </c>
       <c r="H11">
-        <f t="shared" ref="H11:H17" si="18">T11/$X11</f>
+        <f t="shared" ref="H11:H17" si="19">T11/$X11</f>
         <v>0.14620638007734782</v>
       </c>
       <c r="I11">
-        <f t="shared" ref="I11:I17" si="19">U11/$X11</f>
+        <f t="shared" ref="I11:I17" si="20">U11/$X11</f>
         <v>5.5216506829410053E-3</v>
       </c>
       <c r="J11">
-        <f t="shared" ref="J11:J17" si="20">V11/$X11</f>
+        <f t="shared" ref="J11:J17" si="21">V11/$X11</f>
         <v>1.2295173585496168E-4</v>
       </c>
       <c r="K11">
-        <f t="shared" ref="K11:K17" si="21">W11/$X11</f>
+        <f t="shared" ref="K11:K17" si="22">W11/$X11</f>
         <v>0</v>
       </c>
       <c r="L11">
@@ -11276,52 +11526,52 @@
         <v>35.7864</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
       <c r="B12">
-        <f t="shared" ref="B12:B17" si="22">N12/$X12</f>
+        <f t="shared" ref="B12:B17" si="23">N12/$X12</f>
         <v>4.0246143159640146E-2</v>
       </c>
       <c r="C12">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>7.2338864178719889E-2</v>
       </c>
       <c r="D12">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0.14264987620018599</v>
       </c>
       <c r="E12">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0.18757072274443462</v>
       </c>
       <c r="F12">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.21384037106333398</v>
       </c>
       <c r="G12">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0.19464859898943501</v>
       </c>
       <c r="H12">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.14316244104103881</v>
       </c>
       <c r="I12">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>5.411340287036312E-3</v>
       </c>
       <c r="J12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1.2604053463593893E-4</v>
       </c>
       <c r="K12">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>5.6018015393750637E-6</v>
       </c>
       <c r="L12">
-        <f t="shared" ref="L12:L17" si="23">SUM(B12:K12)</f>
+        <f t="shared" ref="L12:L17" si="24">SUM(B12:K12)</f>
         <v>1</v>
       </c>
       <c r="N12">
@@ -11355,56 +11605,56 @@
         <v>2.0000000000000001E-4</v>
       </c>
       <c r="X12">
-        <f t="shared" ref="X12:X17" si="24">SUM(N12:W12)</f>
+        <f t="shared" ref="X12:X17" si="25">SUM(N12:W12)</f>
         <v>35.702799999999996</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13">
+        <f t="shared" si="23"/>
+        <v>4.3399046607525645E-2</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="14"/>
+        <v>7.8329039647039592E-2</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="15"/>
+        <v>0.14166946287786983</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="16"/>
+        <v>0.18148288857398778</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="17"/>
+        <v>0.21248339605165736</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="18"/>
+        <v>0.19317428668883302</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="19"/>
+        <v>0.14397113755417948</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="20"/>
+        <v>5.393683428219641E-3</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="21"/>
+        <v>9.4285468668106829E-5</v>
+      </c>
+      <c r="K13">
         <f t="shared" si="22"/>
-        <v>4.3399046607525645E-2</v>
-      </c>
-      <c r="C13">
-        <f t="shared" si="13"/>
-        <v>7.8329039647039592E-2</v>
-      </c>
-      <c r="D13">
-        <f t="shared" si="14"/>
-        <v>0.14166946287786983</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="15"/>
-        <v>0.18148288857398778</v>
-      </c>
-      <c r="F13">
-        <f t="shared" si="16"/>
-        <v>0.21248339605165736</v>
-      </c>
-      <c r="G13">
-        <f t="shared" si="17"/>
-        <v>0.19317428668883302</v>
-      </c>
-      <c r="H13">
-        <f t="shared" si="18"/>
-        <v>0.14397113755417948</v>
-      </c>
-      <c r="I13">
-        <f t="shared" si="19"/>
-        <v>5.393683428219641E-3</v>
-      </c>
-      <c r="J13">
-        <f t="shared" si="20"/>
-        <v>9.4285468668106829E-5</v>
-      </c>
-      <c r="K13">
-        <f t="shared" si="21"/>
         <v>2.7731020196502011E-6</v>
       </c>
       <c r="L13">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
       <c r="N13">
@@ -11438,56 +11688,56 @@
         <v>1E-4</v>
       </c>
       <c r="X13">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>36.060699999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="B14">
+        <f t="shared" si="23"/>
+        <v>4.3775626664412218E-2</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="14"/>
+        <v>7.793887644249059E-2</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="15"/>
+        <v>0.14178749066520127</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="16"/>
+        <v>0.18137549139789491</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="17"/>
+        <v>0.21157092333488325</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="18"/>
+        <v>0.19615899451888799</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="19"/>
+        <v>0.14157613673190458</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="20"/>
+        <v>5.6981020416789954E-3</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="21"/>
+        <v>1.0990404531428329E-4</v>
+      </c>
+      <c r="K14">
         <f t="shared" si="22"/>
-        <v>4.3775626664412218E-2</v>
-      </c>
-      <c r="C14">
-        <f t="shared" si="13"/>
-        <v>7.793887644249059E-2</v>
-      </c>
-      <c r="D14">
-        <f t="shared" si="14"/>
-        <v>0.14178749066520127</v>
-      </c>
-      <c r="E14">
-        <f t="shared" si="15"/>
-        <v>0.18137549139789491</v>
-      </c>
-      <c r="F14">
-        <f t="shared" si="16"/>
-        <v>0.21157092333488325</v>
-      </c>
-      <c r="G14">
-        <f t="shared" si="17"/>
-        <v>0.19615899451888799</v>
-      </c>
-      <c r="H14">
-        <f t="shared" si="18"/>
-        <v>0.14157613673190458</v>
-      </c>
-      <c r="I14">
-        <f t="shared" si="19"/>
-        <v>5.6981020416789954E-3</v>
-      </c>
-      <c r="J14">
-        <f t="shared" si="20"/>
-        <v>1.0990404531428329E-4</v>
-      </c>
-      <c r="K14">
-        <f t="shared" si="21"/>
         <v>8.4541573318679443E-6</v>
       </c>
       <c r="L14">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
       <c r="N14">
@@ -11521,56 +11771,56 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="X14">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>35.485500000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
       <c r="B15">
+        <f t="shared" si="23"/>
+        <v>4.2773294413103645E-2</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="14"/>
+        <v>6.9477741068348906E-2</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="15"/>
+        <v>0.14183459092425094</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="16"/>
+        <v>0.17931431601212075</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="17"/>
+        <v>0.205220593894579</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="18"/>
+        <v>0.20088482709668959</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="19"/>
+        <v>0.15388123818781482</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="20"/>
+        <v>6.4452128402550718E-3</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="21"/>
+        <v>1.6248435731735475E-4</v>
+      </c>
+      <c r="K15">
         <f t="shared" si="22"/>
-        <v>4.2773294413103645E-2</v>
-      </c>
-      <c r="C15">
-        <f t="shared" si="13"/>
-        <v>6.9477741068348906E-2</v>
-      </c>
-      <c r="D15">
-        <f t="shared" si="14"/>
-        <v>0.14183459092425094</v>
-      </c>
-      <c r="E15">
-        <f t="shared" si="15"/>
-        <v>0.17931431601212075</v>
-      </c>
-      <c r="F15">
-        <f t="shared" si="16"/>
-        <v>0.205220593894579</v>
-      </c>
-      <c r="G15">
-        <f t="shared" si="17"/>
-        <v>0.20088482709668959</v>
-      </c>
-      <c r="H15">
-        <f t="shared" si="18"/>
-        <v>0.15388123818781482</v>
-      </c>
-      <c r="I15">
-        <f t="shared" si="19"/>
-        <v>6.4452128402550718E-3</v>
-      </c>
-      <c r="J15">
-        <f t="shared" si="20"/>
-        <v>1.6248435731735475E-4</v>
-      </c>
-      <c r="K15">
-        <f t="shared" si="21"/>
         <v>5.7012055199071841E-6</v>
       </c>
       <c r="L15">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
       <c r="N15">
@@ -11604,56 +11854,56 @@
         <v>2.0000000000000001E-4</v>
       </c>
       <c r="X15">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>35.080300000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>16</v>
       </c>
       <c r="B16">
+        <f t="shared" si="23"/>
+        <v>4.1800479751657967E-2</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="14"/>
+        <v>7.5055735854381259E-2</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="15"/>
+        <v>0.14603640468463383</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="16"/>
+        <v>0.18119373500776068</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="17"/>
+        <v>0.21734443346973331</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="18"/>
+        <v>0.18988570622266121</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="19"/>
+        <v>0.14285311133060533</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="20"/>
+        <v>5.7090447297869339E-3</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="21"/>
+        <v>1.1006067447438971E-4</v>
+      </c>
+      <c r="K16">
         <f t="shared" si="22"/>
-        <v>4.1800479751657967E-2</v>
-      </c>
-      <c r="C16">
-        <f t="shared" si="13"/>
-        <v>7.5055735854381259E-2</v>
-      </c>
-      <c r="D16">
-        <f t="shared" si="14"/>
-        <v>0.14603640468463383</v>
-      </c>
-      <c r="E16">
-        <f t="shared" si="15"/>
-        <v>0.18119373500776068</v>
-      </c>
-      <c r="F16">
-        <f t="shared" si="16"/>
-        <v>0.21734443346973331</v>
-      </c>
-      <c r="G16">
-        <f t="shared" si="17"/>
-        <v>0.18988570622266121</v>
-      </c>
-      <c r="H16">
-        <f t="shared" si="18"/>
-        <v>0.14285311133060533</v>
-      </c>
-      <c r="I16">
-        <f t="shared" si="19"/>
-        <v>5.7090447297869339E-3</v>
-      </c>
-      <c r="J16">
-        <f t="shared" si="20"/>
-        <v>1.1006067447438971E-4</v>
-      </c>
-      <c r="K16">
-        <f t="shared" si="21"/>
         <v>1.1288274305065613E-5</v>
       </c>
       <c r="L16">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
       <c r="N16">
@@ -11687,7 +11937,7 @@
         <v>4.0000000000000002E-4</v>
       </c>
       <c r="X16">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>35.435000000000002</v>
       </c>
     </row>
@@ -11696,47 +11946,47 @@
         <v>17</v>
       </c>
       <c r="B17">
+        <f t="shared" si="23"/>
+        <v>4.3301022885172347E-2</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="14"/>
+        <v>7.604395113812018E-2</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="15"/>
+        <v>0.14724133505209291</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="16"/>
+        <v>0.18216619512385671</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="17"/>
+        <v>0.21329081077461368</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="18"/>
+        <v>0.18837716728329956</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="19"/>
+        <v>0.14400470984771119</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="20"/>
+        <v>5.4632001294650078E-3</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="21"/>
+        <v>1.088175715266268E-4</v>
+      </c>
+      <c r="K17">
         <f t="shared" si="22"/>
-        <v>4.3301022885172347E-2</v>
-      </c>
-      <c r="C17">
-        <f t="shared" si="13"/>
-        <v>7.604395113812018E-2</v>
-      </c>
-      <c r="D17">
-        <f t="shared" si="14"/>
-        <v>0.14724133505209291</v>
-      </c>
-      <c r="E17">
-        <f t="shared" si="15"/>
-        <v>0.18216619512385671</v>
-      </c>
-      <c r="F17">
-        <f t="shared" si="16"/>
-        <v>0.21329081077461368</v>
-      </c>
-      <c r="G17">
-        <f t="shared" si="17"/>
-        <v>0.18837716728329956</v>
-      </c>
-      <c r="H17">
-        <f t="shared" si="18"/>
-        <v>0.14400470984771119</v>
-      </c>
-      <c r="I17">
-        <f t="shared" si="19"/>
-        <v>5.4632001294650078E-3</v>
-      </c>
-      <c r="J17">
-        <f t="shared" si="20"/>
-        <v>1.088175715266268E-4</v>
-      </c>
-      <c r="K17">
-        <f t="shared" si="21"/>
         <v>2.7901941417083798E-6</v>
       </c>
       <c r="L17">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0.99999999999999989</v>
       </c>
       <c r="N17" s="2">
@@ -11770,7 +12020,7 @@
         <v>1E-4</v>
       </c>
       <c r="X17">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>35.839800000000004</v>
       </c>
     </row>
@@ -12585,15 +12835,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="a4e98822-f433-4c96-8830-5cb2d7491f7d">
@@ -12601,6 +12842,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12623,14 +12873,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E93AF508-606E-42F3-9740-364687CDC244}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2EC63629-1D5E-49FE-AF3E-A7BFE050CE1F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -12638,4 +12880,12 @@
     <ds:schemaRef ds:uri="a4e98822-f433-4c96-8830-5cb2d7491f7d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E93AF508-606E-42F3-9740-364687CDC244}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>